<commit_message>
Modificat pe 26.05.2025 18:13:00
</commit_message>
<xml_diff>
--- a/resurse/bd.xlsx
+++ b/resurse/bd.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Facultate-Ana\Proiect\resurse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F96F193B-F752-4369-BC31-6693756B8528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADF217A9-ECD5-4EC2-B3CB-9543466B9C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="234">
   <si>
     <t>nume</t>
   </si>
@@ -257,9 +257,6 @@
     <t>Consultație pedodontică de specialitate</t>
   </si>
   <si>
-    <t>Anestezie locală computerizată DentaPen</t>
-  </si>
-  <si>
     <t>Inhalosedare cu protoxid de azot pentru copii / ședință</t>
   </si>
   <si>
@@ -297,45 +294,6 @@
   </si>
   <si>
     <t xml:space="preserve">Tratament carie dentară (obturatie)/dinte </t>
-  </si>
-  <si>
-    <t>Aparat dentar fix cu bracketi metalici</t>
-  </si>
-  <si>
-    <t>Aparat dentar fix cu bracketi fizionomici</t>
-  </si>
-  <si>
-    <t>Aparat dentar fix cu bracketi safir</t>
-  </si>
-  <si>
-    <t>Aparat dentar fix sistem DAMON</t>
-  </si>
-  <si>
-    <t>Aparat dentar fix lingual individualizat WIN</t>
-  </si>
-  <si>
-    <t>Aparat dentar fix lingual INCOGNITO</t>
-  </si>
-  <si>
-    <t>Aparat dentar mobil</t>
-  </si>
-  <si>
-    <t>Tratament cu alignere aparat dentar invizibil INVISALIGN Teen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tomografie completă </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tomografie parțială  </t>
-  </si>
-  <si>
-    <t>Inhalosedare cu protoxid de azot pentru copii</t>
-  </si>
-  <si>
-    <t>Sigilare dentară (dinte sănătos, prevenție carii)</t>
-  </si>
-  <si>
-    <t>Tratament carie dentară (obturatie)</t>
   </si>
   <si>
     <t>Evaluare medicală orală și plan de tratament.</t>
@@ -787,7 +745,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="\'\A\i\r\ \F\l\o\w\ \t\o\t\a\l\ \(\ambbe\le\ \a\r\c\ade\)\.\j\pg\'"/>
+    <numFmt numFmtId="164" formatCode="\'\A\i\r\ \F\l\o\w\ \t\o\t\a\l\ \(\ambbe\le\ \a\r\c\ade\)\.\j\pg\'"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -832,7 +790,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -841,9 +799,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -860,7 +815,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1149,7 +1104,7 @@
   <cols>
     <col min="2" max="2" width="86.36328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.453125" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.453125" style="9" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.08984375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="29.90625" style="3" bestFit="1" customWidth="1"/>
@@ -1167,37 +1122,37 @@
     <col min="25" max="25" width="86.36328125" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="57.54296875" customWidth="1"/>
     <col min="28" max="28" width="19.08984375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="10.453125" style="10" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="10.453125" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="A1" s="7"/>
-      <c r="B1" s="7" t="s">
+      <c r="A1" s="6"/>
+      <c r="B1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="G1" s="7" t="s">
+      <c r="E1" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="G1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>205</v>
+      <c r="H1" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>191</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>4</v>
@@ -1208,37 +1163,37 @@
       <c r="R1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="S1" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="T1" s="7" t="s">
+      <c r="S1" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="T1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="U1" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="V1" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="W1" s="7" t="s">
+      <c r="U1" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="V1" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="W1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="Y1" s="7" t="s">
+      <c r="Y1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="AA1" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="AB1" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="AC1" s="9" t="s">
+      <c r="AA1" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="AB1" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="AC1" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="7"/>
-      <c r="B2" s="8" t="str">
+      <c r="A2" s="6"/>
+      <c r="B2" s="7" t="str">
         <f>"(" &amp; "'" &amp; Y2 &amp; "'" &amp; ", "</f>
         <v xml:space="preserve">('Consultație', </v>
       </c>
@@ -1246,7 +1201,7 @@
         <f xml:space="preserve"> "'" &amp; W2 &amp; "'" &amp; ", "</f>
         <v xml:space="preserve">'Evaluare medicală orală și plan de tratament.', </v>
       </c>
-      <c r="D2" s="9" t="str">
+      <c r="D2" s="8" t="str">
         <f xml:space="preserve"> AC2 &amp; ", "</f>
         <v xml:space="preserve">150, </v>
       </c>
@@ -1258,64 +1213,64 @@
         <f xml:space="preserve"> "'" &amp; U2 &amp; "'" &amp; ", "</f>
         <v xml:space="preserve">'Redusă', </v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <f xml:space="preserve"> "'" &amp; T2 &amp; "'" &amp; ", "</f>
         <v xml:space="preserve">'Consult stomatologic', </v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="4" t="str">
         <f xml:space="preserve"> "'" &amp; S2 &amp; "'" &amp; ", "</f>
         <v xml:space="preserve">'Profilaxie și igienizare dentară', </v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <f xml:space="preserve"> AB2 &amp; ", "</f>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="5" t="str">
         <f xml:space="preserve"> "'" &amp; AA2 &amp; "'" &amp;  ", "</f>
         <v xml:space="preserve">'{"Echipamente_evaluare"}', </v>
       </c>
-      <c r="K2" s="11" t="str">
+      <c r="K2" s="10" t="str">
         <f xml:space="preserve"> " ' " &amp; R2 &amp; ".jpg" &amp; " ' " &amp; " ),"</f>
-        <v xml:space="preserve"> ' Air Flow total (ambele arcade).jpg '  ),</v>
+        <v xml:space="preserve"> ' Consultație.jpg '  ),</v>
       </c>
       <c r="L2" s="1"/>
-      <c r="P2" s="7" t="s">
+      <c r="P2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="R2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="S2" s="5" t="s">
+      <c r="R2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="T2" s="6" t="s">
-        <v>162</v>
+      <c r="T2" s="5" t="s">
+        <v>148</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="Y2" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="Y2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="AA2" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="AB2" s="6" t="b">
+      <c r="AA2" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="AB2" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC2" s="9">
+      <c r="AC2" s="8">
         <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="7"/>
-      <c r="B3" s="8" t="str">
+      <c r="A3" s="6"/>
+      <c r="B3" s="7" t="str">
         <f t="shared" ref="B3:B46" si="0">"(" &amp; "'" &amp; Y3 &amp; "'" &amp; ", "</f>
         <v xml:space="preserve">('Detartraj cu ultrasunete + periaj profesional', </v>
       </c>
@@ -1323,7 +1278,7 @@
         <f t="shared" ref="C3:C46" si="1" xml:space="preserve"> "'" &amp; W3 &amp; "'" &amp; ", "</f>
         <v xml:space="preserve">'Curățare completă a tartrului și lustruire dentară.', </v>
       </c>
-      <c r="D3" s="9" t="str">
+      <c r="D3" s="8" t="str">
         <f t="shared" ref="D3:D46" si="2" xml:space="preserve"> AC3 &amp; ", "</f>
         <v xml:space="preserve">350, </v>
       </c>
@@ -1335,64 +1290,64 @@
         <f t="shared" ref="F3:F46" si="4" xml:space="preserve"> "'" &amp; U3 &amp; "'" &amp; ", "</f>
         <v xml:space="preserve">'Redusă', </v>
       </c>
-      <c r="G3" s="6" t="str">
+      <c r="G3" s="5" t="str">
         <f t="shared" ref="G3:G46" si="5" xml:space="preserve"> "'" &amp; T3 &amp; "'" &amp; ", "</f>
         <v xml:space="preserve">'Detartraj complet', </v>
       </c>
-      <c r="H3" s="5" t="str">
+      <c r="H3" s="4" t="str">
         <f t="shared" ref="H3:H46" si="6" xml:space="preserve"> "'" &amp; S3 &amp; "'" &amp; ", "</f>
         <v xml:space="preserve">'Profilaxie și igienizare dentară', </v>
       </c>
-      <c r="I3" s="6" t="str">
+      <c r="I3" s="5" t="str">
         <f t="shared" ref="I3:I46" si="7" xml:space="preserve"> AB3 &amp; ", "</f>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J3" s="6" t="str">
+      <c r="J3" s="5" t="str">
         <f t="shared" ref="J3:J46" si="8" xml:space="preserve"> "'" &amp; AA3 &amp; "'" &amp;  ", "</f>
         <v xml:space="preserve">'{"Perii", "ultrasunete", "gel"}', </v>
       </c>
-      <c r="K3" s="11" t="str">
+      <c r="K3" s="10" t="str">
         <f xml:space="preserve"> "'" &amp; R3 &amp; ".jpg" &amp; "'" &amp; "),"</f>
-        <v>'Albire dentară.jpg'),</v>
+        <v>'Detartraj cu ultrasunete + periaj profesional.jpg'),</v>
       </c>
       <c r="L3" s="1"/>
-      <c r="P3" s="7" t="s">
+      <c r="P3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="R3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="S3" s="5" t="s">
+      <c r="R3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="S3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="T3" s="6" t="s">
-        <v>163</v>
+      <c r="T3" s="5" t="s">
+        <v>149</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="W3" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="Y3" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="AA3" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="AB3" s="6" t="b">
+      <c r="AA3" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="AB3" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC3" s="9">
+      <c r="AC3" s="8">
         <v>350</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8" t="str">
+      <c r="A4" s="6"/>
+      <c r="B4" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Air Flow total (ambele arcade)', </v>
       </c>
@@ -1400,7 +1355,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Curățare cu jet de aer, apă și pulbere, pentru pete și placă.', </v>
       </c>
-      <c r="D4" s="9" t="str">
+      <c r="D4" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">250, </v>
       </c>
@@ -1412,64 +1367,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Redusă', </v>
       </c>
-      <c r="G4" s="6" t="str">
+      <c r="G4" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Air Flow', </v>
       </c>
-      <c r="H4" s="5" t="str">
+      <c r="H4" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Profilaxie și igienizare dentară', </v>
       </c>
-      <c r="I4" s="6" t="str">
+      <c r="I4" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J4" s="6" t="str">
+      <c r="J4" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Aparat_Air_Flow", "pulbere", "apă"}', </v>
       </c>
-      <c r="K4" s="11" t="str">
+      <c r="K4" s="10" t="str">
         <f t="shared" ref="K4:K46" si="9" xml:space="preserve"> "'" &amp; R4 &amp; ".jpg" &amp; "'" &amp; "),"</f>
-        <v>'Anestezie locală computerizată DentaPen.jpg'),</v>
+        <v>'Air Flow total (ambele arcade).jpg'),</v>
       </c>
       <c r="L4" s="1"/>
-      <c r="P4" s="7" t="s">
+      <c r="P4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="R4" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="S4" s="5" t="s">
+      <c r="R4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="S4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="T4" s="6" t="s">
-        <v>164</v>
+      <c r="T4" s="5" t="s">
+        <v>150</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="W4" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="Y4" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="Y4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="AA4" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="AB4" s="6" t="b">
+      <c r="AA4" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="AB4" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC4" s="9">
+      <c r="AC4" s="8">
         <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="7"/>
-      <c r="B5" s="8" t="str">
+      <c r="A5" s="6"/>
+      <c r="B5" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Periaj profesional Happy Brush', </v>
       </c>
@@ -1477,7 +1432,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Periaj specializat pentru igienizare și luciu dentar.', </v>
       </c>
-      <c r="D5" s="9" t="str">
+      <c r="D5" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">150, </v>
       </c>
@@ -1489,64 +1444,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Redusă', </v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Periaj mecanic', </v>
       </c>
-      <c r="H5" s="5" t="str">
+      <c r="H5" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Profilaxie și igienizare dentară', </v>
       </c>
-      <c r="I5" s="6" t="str">
+      <c r="I5" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J5" s="6" t="str">
+      <c r="J5" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Perii_Happy_Brush", "pastă"}', </v>
       </c>
-      <c r="K5" s="11" t="str">
+      <c r="K5" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Aparat dentar fix cu bracketi fizionomici.jpg'),</v>
+        <v>'Periaj profesional Happy Brush.jpg'),</v>
       </c>
       <c r="L5" s="1"/>
-      <c r="P5" s="7" t="s">
+      <c r="P5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="R5" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="S5" s="5" t="s">
+      <c r="R5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="S5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="T5" s="6" t="s">
-        <v>165</v>
+      <c r="T5" s="5" t="s">
+        <v>151</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="Y5" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="AA5" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="AB5" s="6" t="b">
+      <c r="AA5" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="AB5" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC5" s="9">
+      <c r="AC5" s="8">
         <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="7"/>
-      <c r="B6" s="8" t="str">
+      <c r="A6" s="6"/>
+      <c r="B6" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Albire dentară', </v>
       </c>
@@ -1554,7 +1509,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Tratament pentru deschiderea nuanței dinților.', </v>
       </c>
-      <c r="D6" s="9" t="str">
+      <c r="D6" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">1500, </v>
       </c>
@@ -1566,64 +1521,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G6" s="6" t="str">
+      <c r="G6" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Albire dentară', </v>
       </c>
-      <c r="H6" s="5" t="str">
+      <c r="H6" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Estetică dentară', </v>
       </c>
-      <c r="I6" s="6" t="str">
+      <c r="I6" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J6" s="6" t="str">
+      <c r="J6" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Gel_albire", "lampă_UV"}', </v>
       </c>
-      <c r="K6" s="11" t="str">
+      <c r="K6" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Aparat dentar fix cu bracketi metalici.jpg'),</v>
+        <v>'Albire dentară.jpg'),</v>
       </c>
       <c r="L6" s="1"/>
-      <c r="P6" s="7" t="s">
+      <c r="P6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="R6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="S6" s="5" t="s">
+      <c r="R6" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="S6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="T6" s="6" t="s">
+      <c r="T6" s="5" t="s">
         <v>16</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="Y6" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="Y6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="AA6" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="AB6" s="6" t="b">
+      <c r="AA6" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="AB6" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC6" s="9">
+      <c r="AC6" s="8">
         <v>1500</v>
       </c>
     </row>
     <row r="7" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="7"/>
-      <c r="B7" s="8" t="str">
+      <c r="A7" s="6"/>
+      <c r="B7" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Fațete dentare ceramice (E-max)', </v>
       </c>
@@ -1631,7 +1586,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Fațete estetice rezistente, din ceramică presată.', </v>
       </c>
-      <c r="D7" s="9" t="str">
+      <c r="D7" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">1500, </v>
       </c>
@@ -1643,64 +1598,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G7" s="6" t="str">
+      <c r="G7" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Fațete E-max', </v>
       </c>
-      <c r="H7" s="5" t="str">
+      <c r="H7" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Estetică dentară', </v>
       </c>
-      <c r="I7" s="6" t="str">
+      <c r="I7" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J7" s="6" t="str">
+      <c r="J7" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Fațete_E-max", "ciment"}', </v>
       </c>
-      <c r="K7" s="11" t="str">
+      <c r="K7" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Aparat dentar fix cu bracketi safir.jpg'),</v>
+        <v>'Fațete dentare ceramice (E-max).jpg'),</v>
       </c>
       <c r="L7" s="1"/>
-      <c r="P7" s="7" t="s">
+      <c r="P7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="R7" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="S7" s="5" t="s">
+      <c r="R7" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="S7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="T7" s="6" t="s">
-        <v>166</v>
+      <c r="T7" s="5" t="s">
+        <v>152</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="Y7" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="Y7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="AA7" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="AB7" s="6" t="b">
+      <c r="AA7" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="AB7" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC7" s="9">
+      <c r="AC7" s="8">
         <v>1500</v>
       </c>
     </row>
     <row r="8" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="7"/>
-      <c r="B8" s="8" t="str">
+      <c r="A8" s="6"/>
+      <c r="B8" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Fațete dentare Full-Zirconiu', </v>
       </c>
@@ -1708,7 +1663,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Fațete opace, foarte rezistente, din zirconiu integral.', </v>
       </c>
-      <c r="D8" s="9" t="str">
+      <c r="D8" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">1250, </v>
       </c>
@@ -1720,64 +1675,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G8" s="6" t="str">
+      <c r="G8" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Fațete zirconiu', </v>
       </c>
-      <c r="H8" s="5" t="str">
+      <c r="H8" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Estetică dentară', </v>
       </c>
-      <c r="I8" s="6" t="str">
+      <c r="I8" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J8" s="6" t="str">
+      <c r="J8" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Fațete_zirconiu", "ciment"}', </v>
       </c>
-      <c r="K8" s="11" t="str">
+      <c r="K8" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Aparat dentar fix lingual INCOGNITO.jpg'),</v>
+        <v>'Fațete dentare Full-Zirconiu.jpg'),</v>
       </c>
       <c r="L8" s="1"/>
-      <c r="P8" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="R8" s="4" t="s">
+      <c r="P8" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="R8" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="S8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="T8" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="U8" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="V8" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="W8" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="S8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="T8" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="W8" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="Y8" s="8" t="s">
+      <c r="Y8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="AA8" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="AB8" s="6" t="b">
+      <c r="AA8" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="AB8" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC8" s="9">
+      <c r="AC8" s="8">
         <v>1250</v>
       </c>
     </row>
     <row r="9" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="7"/>
-      <c r="B9" s="8" t="str">
+      <c r="A9" s="6"/>
+      <c r="B9" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Fațete dentare Non-Prep', </v>
       </c>
@@ -1785,7 +1740,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Fațete aplicate fără șlefuirea dinților.', </v>
       </c>
-      <c r="D9" s="9" t="str">
+      <c r="D9" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">2500, </v>
       </c>
@@ -1797,64 +1752,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G9" s="6" t="str">
+      <c r="G9" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Fațete non-prep', </v>
       </c>
-      <c r="H9" s="5" t="str">
+      <c r="H9" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Estetică dentară', </v>
       </c>
-      <c r="I9" s="6" t="str">
+      <c r="I9" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J9" s="6" t="str">
+      <c r="J9" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Fațete_compozit", "fatete_ceramic", "ciment"}', </v>
       </c>
-      <c r="K9" s="11" t="str">
+      <c r="K9" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Aparat dentar fix lingual individualizat WIN.jpg'),</v>
+        <v>'Fațete dentare Non-Prep.jpg'),</v>
       </c>
       <c r="L9" s="1"/>
-      <c r="P9" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="R9" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="S9" s="5" t="s">
+      <c r="P9" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="R9" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="S9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="T9" s="6" t="s">
-        <v>168</v>
+      <c r="T9" s="5" t="s">
+        <v>154</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="Y9" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="Y9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="AA9" s="6" t="s">
-        <v>223</v>
-      </c>
-      <c r="AB9" s="6" t="b">
+      <c r="AA9" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="AB9" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC9" s="9">
+      <c r="AC9" s="8">
         <v>2500</v>
       </c>
     </row>
     <row r="10" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="7"/>
-      <c r="B10" s="8" t="str">
+      <c r="A10" s="6"/>
+      <c r="B10" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Implant dentar Megagen, INNO (Coreea)', </v>
       </c>
@@ -1862,7 +1817,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Rădăcină dentară artificială, origine Coreea.', </v>
       </c>
-      <c r="D10" s="9" t="str">
+      <c r="D10" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">2700, </v>
       </c>
@@ -1874,64 +1829,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G10" s="6" t="str">
+      <c r="G10" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Implant Megagen', </v>
       </c>
-      <c r="H10" s="5" t="str">
+      <c r="H10" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Implantologie', </v>
       </c>
-      <c r="I10" s="6" t="str">
+      <c r="I10" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J10" s="6" t="str">
+      <c r="J10" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Implant", "șuruburi", "abutment", "kit_chirurgical"}', </v>
       </c>
-      <c r="K10" s="11" t="str">
+      <c r="K10" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Aparat dentar fix sistem DAMON.jpg'),</v>
+        <v>'Implant dentar Megagen, INNO (Coreea).jpg'),</v>
       </c>
       <c r="L10" s="1"/>
-      <c r="P10" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="R10" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="S10" s="7" t="s">
+      <c r="P10" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="R10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="S10" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="T10" s="6" t="s">
-        <v>169</v>
+      <c r="T10" s="5" t="s">
+        <v>155</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="W10" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="Y10" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y10" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="AA10" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="AB10" s="6" t="b">
+      <c r="AA10" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="AB10" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC10" s="9">
+      <c r="AC10" s="8">
         <v>2700</v>
       </c>
     </row>
     <row r="11" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="7"/>
-      <c r="B11" s="8" t="str">
+      <c r="A11" s="6"/>
+      <c r="B11" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Implant dentar ICX (Germania &amp; Elveția)', </v>
       </c>
@@ -1939,7 +1894,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Implant premium german-elvețian.', </v>
       </c>
-      <c r="D11" s="9" t="str">
+      <c r="D11" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">3200, </v>
       </c>
@@ -1951,64 +1906,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G11" s="6" t="str">
+      <c r="G11" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Implant ICX', </v>
       </c>
-      <c r="H11" s="5" t="str">
+      <c r="H11" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Implantologie', </v>
       </c>
-      <c r="I11" s="6" t="str">
+      <c r="I11" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J11" s="6" t="str">
+      <c r="J11" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Implant", "șuruburi", "abutment", "kit_chirurgical"}', </v>
       </c>
-      <c r="K11" s="11" t="str">
+      <c r="K11" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Aparat dentar mobil.jpg'),</v>
+        <v>'Implant dentar ICX (Germania &amp; Elveția).jpg'),</v>
       </c>
       <c r="L11" s="1"/>
-      <c r="P11" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="R11" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="S11" s="7" t="s">
+      <c r="P11" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="R11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="S11" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="T11" s="6" t="s">
-        <v>170</v>
+      <c r="T11" s="5" t="s">
+        <v>156</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="Y11" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y11" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="AA11" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="AB11" s="6" t="b">
+      <c r="AA11" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="AB11" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC11" s="9">
+      <c r="AC11" s="8">
         <v>3200</v>
       </c>
     </row>
     <row r="12" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="7"/>
-      <c r="B12" s="8" t="str">
+      <c r="A12" s="6"/>
+      <c r="B12" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Implant dentar Nobel (SUA)', </v>
       </c>
@@ -2016,7 +1971,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Implant de top, fabricat în SUA.', </v>
       </c>
-      <c r="D12" s="9" t="str">
+      <c r="D12" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">5000, </v>
       </c>
@@ -2028,64 +1983,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G12" s="6" t="str">
+      <c r="G12" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Implant Nobel', </v>
       </c>
-      <c r="H12" s="5" t="str">
+      <c r="H12" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Implantologie', </v>
       </c>
-      <c r="I12" s="6" t="str">
+      <c r="I12" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J12" s="6" t="str">
+      <c r="J12" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Implant", "șuruburi", "abutment", "kit_chirurgical"}', </v>
       </c>
-      <c r="K12" s="11" t="str">
+      <c r="K12" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Bont individualizat.jpg'),</v>
+        <v>'Implant dentar Nobel (SUA).jpg'),</v>
       </c>
       <c r="L12" s="1"/>
-      <c r="P12" s="7" t="s">
+      <c r="P12" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="R12" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="S12" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T12" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="U12" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="V12" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="W12" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y12" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA12" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="R12" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="S12" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="T12" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="U12" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="V12" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="W12" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="Y12" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="AA12" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="AB12" s="6" t="b">
+      <c r="AB12" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC12" s="9">
+      <c r="AC12" s="8">
         <v>5000</v>
       </c>
     </row>
     <row r="13" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="7"/>
-      <c r="B13" s="8" t="str">
+      <c r="A13" s="6"/>
+      <c r="B13" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Bont protetic drept', </v>
       </c>
@@ -2093,7 +2048,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Piesă care susține coroana pe implant, fără unghi.', </v>
       </c>
-      <c r="D13" s="9" t="str">
+      <c r="D13" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">250, </v>
       </c>
@@ -2105,64 +2060,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G13" s="6" t="str">
+      <c r="G13" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Bont drept', </v>
       </c>
-      <c r="H13" s="5" t="str">
+      <c r="H13" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Implantologie', </v>
       </c>
-      <c r="I13" s="6" t="str">
+      <c r="I13" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J13" s="6" t="str">
+      <c r="J13" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Bont_metal", "ciment"}', </v>
       </c>
-      <c r="K13" s="11" t="str">
+      <c r="K13" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Bont protetic angulat.jpg'),</v>
+        <v>'Bont protetic drept.jpg'),</v>
       </c>
       <c r="L13" s="1"/>
-      <c r="P13" s="7" t="s">
+      <c r="P13" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="R13" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="S13" s="7" t="s">
+      <c r="R13" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="S13" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="T13" s="6" t="s">
-        <v>172</v>
+      <c r="T13" s="5" t="s">
+        <v>158</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="W13" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="Y13" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="Y13" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AA13" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="AB13" s="6" t="b">
+      <c r="AA13" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="AB13" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC13" s="9">
+      <c r="AC13" s="8">
         <v>250</v>
       </c>
     </row>
     <row r="14" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="7"/>
-      <c r="B14" s="8" t="str">
+      <c r="A14" s="6"/>
+      <c r="B14" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Bont protetic angulat', </v>
       </c>
@@ -2170,7 +2125,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Piesă pe implant cu înclinație pentru aliniere.', </v>
       </c>
-      <c r="D14" s="9" t="str">
+      <c r="D14" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">500, </v>
       </c>
@@ -2182,64 +2137,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G14" s="6" t="str">
+      <c r="G14" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Bont angulat', </v>
       </c>
-      <c r="H14" s="5" t="str">
+      <c r="H14" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Implantologie', </v>
       </c>
-      <c r="I14" s="6" t="str">
+      <c r="I14" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J14" s="6" t="str">
+      <c r="J14" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Bont_metal", "ciment"}', </v>
       </c>
-      <c r="K14" s="11" t="str">
+      <c r="K14" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Bont protetic din zirconiu.jpg'),</v>
+        <v>'Bont protetic angulat.jpg'),</v>
       </c>
       <c r="L14" s="1"/>
-      <c r="P14" s="7" t="s">
+      <c r="P14" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="R14" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="S14" s="7" t="s">
+      <c r="R14" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S14" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="T14" s="6" t="s">
-        <v>173</v>
+      <c r="T14" s="5" t="s">
+        <v>159</v>
       </c>
       <c r="U14" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="W14" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="Y14" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y14" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA14" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="AB14" s="6" t="b">
+      <c r="AA14" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="AB14" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC14" s="9">
+      <c r="AC14" s="8">
         <v>500</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="7"/>
-      <c r="B15" s="8" t="str">
+      <c r="A15" s="6"/>
+      <c r="B15" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Bont individualizat', </v>
       </c>
@@ -2247,7 +2202,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Piesă personalizată pentru restaurări precise.', </v>
       </c>
-      <c r="D15" s="9" t="str">
+      <c r="D15" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">750, </v>
       </c>
@@ -2259,64 +2214,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G15" s="6" t="str">
+      <c r="G15" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Bont personalizat', </v>
       </c>
-      <c r="H15" s="5" t="str">
+      <c r="H15" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Implantologie', </v>
       </c>
-      <c r="I15" s="6" t="str">
+      <c r="I15" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J15" s="6" t="str">
+      <c r="J15" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Bont_personalizat", "ciment"}', </v>
       </c>
-      <c r="K15" s="11" t="str">
+      <c r="K15" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Bont protetic drept.jpg'),</v>
+        <v>'Bont individualizat.jpg'),</v>
       </c>
       <c r="L15" s="1"/>
-      <c r="P15" s="7" t="s">
+      <c r="P15" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R15" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="S15" s="7" t="s">
+      <c r="R15" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="S15" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="T15" s="6" t="s">
-        <v>174</v>
+      <c r="T15" s="5" t="s">
+        <v>160</v>
       </c>
       <c r="U15" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V15" s="1" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="Y15" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="Y15" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="AA15" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="AB15" s="6" t="b">
+      <c r="AA15" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="AB15" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC15" s="9">
+      <c r="AC15" s="8">
         <v>750</v>
       </c>
     </row>
     <row r="16" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="7"/>
-      <c r="B16" s="8" t="str">
+      <c r="A16" s="6"/>
+      <c r="B16" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Bont protetic din zirconiu', </v>
       </c>
@@ -2324,7 +2279,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Bont estetic, alb, din zirconiu.', </v>
       </c>
-      <c r="D16" s="9" t="str">
+      <c r="D16" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">1000, </v>
       </c>
@@ -2336,64 +2291,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G16" s="6" t="str">
+      <c r="G16" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Bont zirconiu', </v>
       </c>
-      <c r="H16" s="5" t="str">
+      <c r="H16" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Implantologie', </v>
       </c>
-      <c r="I16" s="6" t="str">
+      <c r="I16" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J16" s="6" t="str">
+      <c r="J16" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Bont_zirconiu", "ciment"}', </v>
       </c>
-      <c r="K16" s="11" t="str">
+      <c r="K16" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Consultație.jpg'),</v>
+        <v>'Bont protetic din zirconiu.jpg'),</v>
       </c>
       <c r="L16" s="1"/>
-      <c r="P16" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="R16" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="S16" s="7" t="s">
+      <c r="P16" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="R16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="S16" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="T16" s="6" t="s">
-        <v>175</v>
+      <c r="T16" s="5" t="s">
+        <v>161</v>
       </c>
       <c r="U16" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V16" s="1" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y16" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y16" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="AA16" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="AB16" s="6" t="b">
+      <c r="AA16" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="AB16" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC16" s="9">
+      <c r="AC16" s="8">
         <v>1000</v>
       </c>
     </row>
     <row r="17" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="7"/>
-      <c r="B17" s="8" t="str">
+      <c r="A17" s="6"/>
+      <c r="B17" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Aparat dentar fix cu bracketi metalici / arcadă', </v>
       </c>
@@ -2401,7 +2356,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Corecție ortodontică clasică, cu metal.', </v>
       </c>
-      <c r="D17" s="9" t="str">
+      <c r="D17" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">4800, </v>
       </c>
@@ -2413,64 +2368,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G17" s="6" t="str">
+      <c r="G17" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Aparat fix', </v>
       </c>
-      <c r="H17" s="5" t="str">
+      <c r="H17" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Ortodonție', </v>
       </c>
-      <c r="I17" s="6" t="str">
+      <c r="I17" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J17" s="6" t="str">
+      <c r="J17" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Bracketi_metalici", "arcuri_linguale"}', </v>
       </c>
-      <c r="K17" s="11" t="str">
+      <c r="K17" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Consultație pedodontică de specialitate.jpg'),</v>
+        <v>'Aparat dentar fix cu bracketi metalici / arcadă.jpg'),</v>
       </c>
       <c r="L17" s="1"/>
-      <c r="P17" s="7" t="s">
+      <c r="P17" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="R17" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="S17" s="7" t="s">
+      <c r="R17" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="S17" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="T17" s="6" t="s">
-        <v>197</v>
+      <c r="T17" s="5" t="s">
+        <v>183</v>
       </c>
       <c r="U17" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V17" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="W17" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="Y17" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="Y17" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="AA17" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="AB17" s="6" t="b">
+      <c r="AA17" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="AB17" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC17" s="9">
+      <c r="AC17" s="8">
         <v>4800</v>
       </c>
     </row>
     <row r="18" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="7"/>
-      <c r="B18" s="8" t="str">
+      <c r="A18" s="6"/>
+      <c r="B18" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Aparat dentar fix cu bracketi fizionomici / arcadă', </v>
       </c>
@@ -2478,7 +2433,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Bracketi colorați în nuanța dinților.', </v>
       </c>
-      <c r="D18" s="9" t="str">
+      <c r="D18" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">4900, </v>
       </c>
@@ -2490,64 +2445,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G18" s="6" t="str">
+      <c r="G18" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Aparat fix', </v>
       </c>
-      <c r="H18" s="5" t="str">
+      <c r="H18" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Ortodonție', </v>
       </c>
-      <c r="I18" s="6" t="str">
+      <c r="I18" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J18" s="6" t="str">
+      <c r="J18" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Bracketi_fizionomici", "arcuri_linguale"}', </v>
       </c>
-      <c r="K18" s="11" t="str">
+      <c r="K18" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Consultație stomatologie pediatrică.jpg'),</v>
+        <v>'Aparat dentar fix cu bracketi fizionomici / arcadă.jpg'),</v>
       </c>
       <c r="L18" s="1"/>
-      <c r="P18" s="7" t="s">
+      <c r="P18" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="R18" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="S18" s="7" t="s">
+      <c r="R18" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="S18" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="T18" s="6" t="s">
-        <v>197</v>
+      <c r="T18" s="5" t="s">
+        <v>183</v>
       </c>
       <c r="U18" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V18" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="W18" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="Y18" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="Y18" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="AA18" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="AB18" s="6" t="b">
+      <c r="AA18" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="AB18" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC18" s="9">
+      <c r="AC18" s="8">
         <v>4900</v>
       </c>
     </row>
     <row r="19" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="7"/>
-      <c r="B19" s="8" t="str">
+      <c r="A19" s="6"/>
+      <c r="B19" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Aparat dentar fix cu bracketi safir / arcadă', </v>
       </c>
@@ -2555,7 +2510,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Bracketi transparenți, din safir.', </v>
       </c>
-      <c r="D19" s="9" t="str">
+      <c r="D19" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">6300, </v>
       </c>
@@ -2567,64 +2522,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G19" s="6" t="str">
+      <c r="G19" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Aparat fix', </v>
       </c>
-      <c r="H19" s="5" t="str">
+      <c r="H19" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Ortodonție', </v>
       </c>
-      <c r="I19" s="6" t="str">
+      <c r="I19" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J19" s="6" t="str">
+      <c r="J19" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Bracketi_safir", "arcuri_linguale"}', </v>
       </c>
-      <c r="K19" s="11" t="str">
+      <c r="K19" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Detartraj cu ultrasunete + periaj profesional.jpg'),</v>
+        <v>'Aparat dentar fix cu bracketi safir / arcadă.jpg'),</v>
       </c>
       <c r="L19" s="1"/>
-      <c r="P19" s="7" t="s">
+      <c r="P19" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="R19" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="S19" s="7" t="s">
+      <c r="R19" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S19" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="T19" s="6" t="s">
-        <v>197</v>
+      <c r="T19" s="5" t="s">
+        <v>183</v>
       </c>
       <c r="U19" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V19" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="W19" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="Y19" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="Y19" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AA19" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="AB19" s="6" t="b">
+      <c r="AA19" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="AB19" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC19" s="9">
+      <c r="AC19" s="8">
         <v>6300</v>
       </c>
     </row>
     <row r="20" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="7"/>
-      <c r="B20" s="8" t="str">
+      <c r="A20" s="6"/>
+      <c r="B20" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Aparat dentar fix sistem DAMON / arcadă: ', </v>
       </c>
@@ -2632,7 +2587,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Sistem cu frecare redusă, confort crescut.', </v>
       </c>
-      <c r="D20" s="9" t="str">
+      <c r="D20" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">6300, </v>
       </c>
@@ -2644,64 +2599,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G20" s="6" t="str">
+      <c r="G20" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Aparat fix', </v>
       </c>
-      <c r="H20" s="5" t="str">
+      <c r="H20" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Ortodonție', </v>
       </c>
-      <c r="I20" s="6" t="str">
+      <c r="I20" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J20" s="6" t="str">
+      <c r="J20" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Bracketi_DAMON", "arcuri_linguale"}', </v>
       </c>
-      <c r="K20" s="11" t="str">
+      <c r="K20" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Drenaj abces.jpg'),</v>
+        <v>'Aparat dentar fix sistem DAMON / arcadă: .jpg'),</v>
       </c>
       <c r="L20" s="1"/>
-      <c r="P20" s="7" t="s">
+      <c r="P20" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="R20" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="S20" s="7" t="s">
+      <c r="R20" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="S20" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="T20" s="6" t="s">
-        <v>197</v>
+      <c r="T20" s="5" t="s">
+        <v>183</v>
       </c>
       <c r="U20" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V20" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="W20" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="Y20" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA20" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="AB20" s="6" t="b">
+        <v>104</v>
+      </c>
+      <c r="Y20" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AA20" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB20" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC20" s="9">
+      <c r="AC20" s="8">
         <v>6300</v>
       </c>
     </row>
     <row r="21" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="7"/>
-      <c r="B21" s="8" t="str">
+      <c r="A21" s="6"/>
+      <c r="B21" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Aparat dentar fix lingual individualizat WIN / arcadă: ', </v>
       </c>
@@ -2709,7 +2664,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Aparat invizibil, montat pe interior.', </v>
       </c>
-      <c r="D21" s="9" t="str">
+      <c r="D21" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">9000, </v>
       </c>
@@ -2721,64 +2676,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G21" s="6" t="str">
+      <c r="G21" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Aparat lingual', </v>
       </c>
-      <c r="H21" s="5" t="str">
+      <c r="H21" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Ortodonție', </v>
       </c>
-      <c r="I21" s="6" t="str">
+      <c r="I21" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J21" s="6" t="str">
+      <c r="J21" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Bracketi_WIN", "arcuri_linguale"}', </v>
       </c>
-      <c r="K21" s="11" t="str">
+      <c r="K21" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Extracție dinte monoradicular.jpg'),</v>
+        <v>'Aparat dentar fix lingual individualizat WIN / arcadă: .jpg'),</v>
       </c>
       <c r="L21" s="1"/>
-      <c r="P21" s="7" t="s">
+      <c r="P21" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="R21" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="S21" s="7" t="s">
+      <c r="R21" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="S21" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="T21" s="6" t="s">
-        <v>198</v>
+      <c r="T21" s="5" t="s">
+        <v>184</v>
       </c>
       <c r="U21" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V21" s="1" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="W21" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="Y21" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="AA21" s="6" t="s">
-        <v>243</v>
-      </c>
-      <c r="AB21" s="6" t="b">
+        <v>105</v>
+      </c>
+      <c r="Y21" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AA21" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="AB21" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC21" s="9">
+      <c r="AC21" s="8">
         <v>9000</v>
       </c>
     </row>
     <row r="22" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="7"/>
-      <c r="B22" s="8" t="str">
+      <c r="A22" s="6"/>
+      <c r="B22" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Aparat dentar fix lingual INCOGNITO / arcadă: ', </v>
       </c>
@@ -2786,7 +2741,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Ortodonție invizibilă de lux, internă.', </v>
       </c>
-      <c r="D22" s="9" t="str">
+      <c r="D22" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">12000, </v>
       </c>
@@ -2798,64 +2753,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G22" s="6" t="str">
+      <c r="G22" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Aparat lingual', </v>
       </c>
-      <c r="H22" s="5" t="str">
+      <c r="H22" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Ortodonție', </v>
       </c>
-      <c r="I22" s="6" t="str">
+      <c r="I22" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J22" s="6" t="str">
+      <c r="J22" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Bracketi_INCOGNITO", "arcuri_linguale"}', </v>
       </c>
-      <c r="K22" s="11" t="str">
+      <c r="K22" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Extracție dinte pluriradicular.jpg'),</v>
+        <v>'Aparat dentar fix lingual INCOGNITO / arcadă: .jpg'),</v>
       </c>
       <c r="L22" s="1"/>
-      <c r="P22" s="7" t="s">
+      <c r="P22" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="R22" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="S22" s="7" t="s">
+      <c r="R22" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="S22" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="T22" s="6" t="s">
-        <v>198</v>
+      <c r="T22" s="5" t="s">
+        <v>184</v>
       </c>
       <c r="U22" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V22" s="1" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="W22" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="Y22" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA22" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="AB22" s="6" t="b">
+        <v>106</v>
+      </c>
+      <c r="Y22" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA22" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="AB22" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC22" s="9">
+      <c r="AC22" s="8">
         <v>12000</v>
       </c>
     </row>
     <row r="23" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="7"/>
-      <c r="B23" s="8" t="str">
+      <c r="A23" s="6"/>
+      <c r="B23" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Aparat dentar mobil / arcadă', </v>
       </c>
@@ -2863,7 +2818,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Dispozitiv detașabil pentru copii sau corecții minore.', </v>
       </c>
-      <c r="D23" s="9" t="str">
+      <c r="D23" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">1850, </v>
       </c>
@@ -2875,64 +2830,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Redusă', </v>
       </c>
-      <c r="G23" s="6" t="str">
+      <c r="G23" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Aparat mobil', </v>
       </c>
-      <c r="H23" s="5" t="str">
+      <c r="H23" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Ortodonție', </v>
       </c>
-      <c r="I23" s="6" t="str">
+      <c r="I23" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J23" s="6" t="str">
+      <c r="J23" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Aliniatori", "arcuri", "suporturi"}', </v>
       </c>
-      <c r="K23" s="11" t="str">
+      <c r="K23" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Extracție dinte temporar.jpg'),</v>
+        <v>'Aparat dentar mobil / arcadă.jpg'),</v>
       </c>
       <c r="L23" s="1"/>
-      <c r="P23" s="7" t="s">
+      <c r="P23" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="R23" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="S23" s="7" t="s">
+      <c r="R23" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="S23" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="T23" s="6" t="s">
-        <v>199</v>
+      <c r="T23" s="5" t="s">
+        <v>185</v>
       </c>
       <c r="U23" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="V23" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="W23" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="Y23" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA23" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="V23" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="W23" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="Y23" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="AA23" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="AB23" s="6" t="b">
+      <c r="AB23" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC23" s="9">
+      <c r="AC23" s="8">
         <v>1850</v>
       </c>
     </row>
     <row r="24" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="7"/>
-      <c r="B24" s="8" t="str">
+      <c r="A24" s="6"/>
+      <c r="B24" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Tratament cu alignere aparat INVISALIGN LITE', </v>
       </c>
@@ -2940,7 +2895,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Gutieră transparentă pentru corecții minore.', </v>
       </c>
-      <c r="D24" s="9" t="str">
+      <c r="D24" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">10000, </v>
       </c>
@@ -2952,64 +2907,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G24" s="6" t="str">
+      <c r="G24" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Invisalign Lite', </v>
       </c>
-      <c r="H24" s="5" t="str">
+      <c r="H24" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Ortodonție', </v>
       </c>
-      <c r="I24" s="6" t="str">
+      <c r="I24" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J24" s="6" t="str">
+      <c r="J24" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Aliniatori_Invisalign", "materiale_imobilizare"}', </v>
       </c>
-      <c r="K24" s="11" t="str">
+      <c r="K24" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Extracție molar de minte.jpg'),</v>
+        <v>'Tratament cu alignere aparat INVISALIGN LITE.jpg'),</v>
       </c>
       <c r="L24" s="1"/>
-      <c r="P24" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="R24" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="S24" s="7" t="s">
+      <c r="P24" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="R24" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="S24" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="T24" s="6" t="s">
-        <v>176</v>
+      <c r="T24" s="5" t="s">
+        <v>162</v>
       </c>
       <c r="U24" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V24" s="1" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="W24" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="Y24" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="Y24" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="AA24" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="AB24" s="6" t="b">
+      <c r="AA24" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="AB24" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC24" s="9">
+      <c r="AC24" s="8">
         <v>10000</v>
       </c>
     </row>
     <row r="25" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A25" s="7"/>
-      <c r="B25" s="8" t="str">
+      <c r="A25" s="6"/>
+      <c r="B25" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Tratament cu alignere aparat dentar invizibil INVISALIGN Teen / ambele arcade', </v>
       </c>
@@ -3017,7 +2972,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Aliniatori transparenți pentru adolescenți.', </v>
       </c>
-      <c r="D25" s="9" t="str">
+      <c r="D25" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">15000, </v>
       </c>
@@ -3029,64 +2984,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G25" s="6" t="str">
+      <c r="G25" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Invisalign Teen', </v>
       </c>
-      <c r="H25" s="5" t="str">
+      <c r="H25" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Ortodonție', </v>
       </c>
-      <c r="I25" s="6" t="str">
+      <c r="I25" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J25" s="6" t="str">
+      <c r="J25" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Aliniatori_Invisalign_Teen", "materiale imobilizare"}', </v>
       </c>
-      <c r="K25" s="11" t="str">
+      <c r="K25" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Fațete dentare ceramice (E-max).jpg'),</v>
+        <v>'Tratament cu alignere aparat dentar invizibil INVISALIGN Teen / ambele arcade.jpg'),</v>
       </c>
       <c r="L25" s="1"/>
-      <c r="P25" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="R25" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="S25" s="7" t="s">
+      <c r="P25" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="R25" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="S25" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="T25" s="6" t="s">
-        <v>177</v>
+      <c r="T25" s="5" t="s">
+        <v>163</v>
       </c>
       <c r="U25" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V25" s="1" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="W25" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Y25" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="Y25" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="AA25" s="6" t="s">
-        <v>246</v>
-      </c>
-      <c r="AB25" s="6" t="b">
+      <c r="AA25" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="AB25" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC25" s="9">
+      <c r="AC25" s="8">
         <v>15000</v>
       </c>
     </row>
     <row r="26" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A26" s="7"/>
-      <c r="B26" s="8" t="str">
+      <c r="A26" s="6"/>
+      <c r="B26" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Tratament endodontic dinte monoradicular​', </v>
       </c>
@@ -3094,7 +3049,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Curățare și sigilare canal la dinte cu o rădăcină.', </v>
       </c>
-      <c r="D26" s="9" t="str">
+      <c r="D26" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">200, </v>
       </c>
@@ -3106,64 +3061,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G26" s="6" t="str">
+      <c r="G26" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Endo monoradicular', </v>
       </c>
-      <c r="H26" s="5" t="str">
+      <c r="H26" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Endodonție', </v>
       </c>
-      <c r="I26" s="6" t="str">
+      <c r="I26" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J26" s="6" t="str">
+      <c r="J26" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"conuri", "instrumente_endodontice", "pastă"}', </v>
       </c>
-      <c r="K26" s="11" t="str">
+      <c r="K26" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Fațete dentare Full-Zirconiu.jpg'),</v>
+        <v>'Tratament endodontic dinte monoradicular​.jpg'),</v>
       </c>
       <c r="L26" s="1"/>
-      <c r="P26" s="7" t="s">
+      <c r="P26" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="R26" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="S26" s="7" t="s">
+      <c r="R26" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="S26" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="T26" s="6" t="s">
-        <v>178</v>
+      <c r="T26" s="5" t="s">
+        <v>164</v>
       </c>
       <c r="U26" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V26" s="1" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="W26" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="Y26" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="AA26" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="AB26" s="6" t="b">
+        <v>110</v>
+      </c>
+      <c r="Y26" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="AA26" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="AB26" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC26" s="9">
+      <c r="AC26" s="8">
         <v>200</v>
       </c>
     </row>
     <row r="27" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="7"/>
-      <c r="B27" s="8" t="str">
+      <c r="A27" s="6"/>
+      <c r="B27" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Tratament endodontic premolar', </v>
       </c>
@@ -3171,7 +3126,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Tratament de canal pentru premolar.', </v>
       </c>
-      <c r="D27" s="9" t="str">
+      <c r="D27" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">250, </v>
       </c>
@@ -3183,64 +3138,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G27" s="6" t="str">
+      <c r="G27" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Endo premolar', </v>
       </c>
-      <c r="H27" s="5" t="str">
+      <c r="H27" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Endodonție', </v>
       </c>
-      <c r="I27" s="6" t="str">
+      <c r="I27" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J27" s="6" t="str">
+      <c r="J27" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"conuri", "instrumente_endodontice", "pastă"}', </v>
       </c>
-      <c r="K27" s="11" t="str">
+      <c r="K27" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Fațete dentare Non-Prep.jpg'),</v>
+        <v>'Tratament endodontic premolar.jpg'),</v>
       </c>
       <c r="L27" s="1"/>
-      <c r="P27" s="7" t="s">
+      <c r="P27" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="R27" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="S27" s="7" t="s">
+      <c r="R27" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="S27" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="T27" s="6" t="s">
-        <v>179</v>
+      <c r="T27" s="5" t="s">
+        <v>165</v>
       </c>
       <c r="U27" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V27" s="1" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
       <c r="W27" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="Y27" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="Y27" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="AA27" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="AB27" s="6" t="b">
+      <c r="AA27" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="AB27" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC27" s="9">
+      <c r="AC27" s="8">
         <v>250</v>
       </c>
     </row>
     <row r="28" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="7"/>
-      <c r="B28" s="8" t="str">
+      <c r="A28" s="6"/>
+      <c r="B28" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Tratament endodontic dinte pluriradicular', </v>
       </c>
@@ -3248,7 +3203,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Curățare canale pentru molari.', </v>
       </c>
-      <c r="D28" s="9" t="str">
+      <c r="D28" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">350, </v>
       </c>
@@ -3260,64 +3215,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G28" s="6" t="str">
+      <c r="G28" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Endo pluriradicular', </v>
       </c>
-      <c r="H28" s="5" t="str">
+      <c r="H28" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Endodonție', </v>
       </c>
-      <c r="I28" s="6" t="str">
+      <c r="I28" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J28" s="6" t="str">
+      <c r="J28" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"conuri", "instrumente_endodontice", "pastă"}', </v>
       </c>
-      <c r="K28" s="11" t="str">
+      <c r="K28" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Implant dentar ICX (Germania &amp; Elveția).jpg'),</v>
+        <v>'Tratament endodontic dinte pluriradicular.jpg'),</v>
       </c>
       <c r="L28" s="1"/>
-      <c r="P28" s="7" t="s">
+      <c r="P28" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="R28" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="S28" s="7" t="s">
+      <c r="R28" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="S28" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="T28" s="6" t="s">
-        <v>180</v>
+      <c r="T28" s="5" t="s">
+        <v>166</v>
       </c>
       <c r="U28" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V28" s="1" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="W28" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="Y28" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="Y28" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="AA28" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="AB28" s="6" t="b">
+      <c r="AA28" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="AB28" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC28" s="9">
+      <c r="AC28" s="8">
         <v>350</v>
       </c>
     </row>
     <row r="29" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A29" s="7"/>
-      <c r="B29" s="8" t="str">
+      <c r="A29" s="6"/>
+      <c r="B29" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Retratament endodontic', </v>
       </c>
@@ -3325,7 +3280,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Refacere tratament canal anterior.', </v>
       </c>
-      <c r="D29" s="9" t="str">
+      <c r="D29" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">350, </v>
       </c>
@@ -3337,64 +3292,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G29" s="6" t="str">
+      <c r="G29" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Endo refacere', </v>
       </c>
-      <c r="H29" s="5" t="str">
+      <c r="H29" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Endodonție', </v>
       </c>
-      <c r="I29" s="6" t="str">
+      <c r="I29" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J29" s="6" t="str">
+      <c r="J29" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"conuri", "instrumente_endodontice", "pastă"}', </v>
       </c>
-      <c r="K29" s="11" t="str">
+      <c r="K29" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Implant dentar Megagen, INNO (Coreea).jpg'),</v>
+        <v>'Retratament endodontic.jpg'),</v>
       </c>
       <c r="L29" s="1"/>
-      <c r="P29" s="7" t="s">
+      <c r="P29" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="R29" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="S29" s="7" t="s">
+      <c r="R29" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="S29" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="T29" s="6" t="s">
-        <v>181</v>
+      <c r="T29" s="5" t="s">
+        <v>167</v>
       </c>
       <c r="U29" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V29" s="1" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="W29" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="Y29" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="Y29" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="AA29" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="AB29" s="6" t="b">
+      <c r="AA29" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="AB29" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC29" s="9">
+      <c r="AC29" s="8">
         <v>350</v>
       </c>
     </row>
     <row r="30" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A30" s="7"/>
-      <c r="B30" s="8" t="str">
+      <c r="A30" s="6"/>
+      <c r="B30" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Utilizarea microscopului ​', </v>
       </c>
@@ -3402,7 +3357,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Precizie maximă în tratamente dentare.', </v>
       </c>
-      <c r="D30" s="9" t="str">
+      <c r="D30" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">200, </v>
       </c>
@@ -3414,64 +3369,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G30" s="6" t="str">
+      <c r="G30" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Microscop endo', </v>
       </c>
-      <c r="H30" s="5" t="str">
+      <c r="H30" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Endodonție', </v>
       </c>
-      <c r="I30" s="6" t="str">
+      <c r="I30" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J30" s="6" t="str">
+      <c r="J30" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Microscop_dentar", "instrumente_chirurgicale"}', </v>
       </c>
-      <c r="K30" s="11" t="str">
+      <c r="K30" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Implant dentar Nobel (SUA).jpg'),</v>
+        <v>'Utilizarea microscopului ​.jpg'),</v>
       </c>
       <c r="L30" s="1"/>
-      <c r="P30" s="7" t="s">
+      <c r="P30" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="R30" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="S30" s="7" t="s">
+      <c r="R30" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="S30" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="T30" s="6" t="s">
-        <v>182</v>
+      <c r="T30" s="5" t="s">
+        <v>168</v>
       </c>
       <c r="U30" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V30" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="W30" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="Y30" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="AA30" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="AB30" s="6" t="b">
+        <v>114</v>
+      </c>
+      <c r="Y30" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="AA30" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="AB30" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC30" s="9">
+      <c r="AC30" s="8">
         <v>200</v>
       </c>
     </row>
     <row r="31" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="7"/>
-      <c r="B31" s="8" t="str">
+      <c r="A31" s="6"/>
+      <c r="B31" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Radiografie locală', </v>
       </c>
@@ -3479,7 +3434,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Imagine a unei zone restrânse dentare.', </v>
       </c>
-      <c r="D31" s="9" t="str">
+      <c r="D31" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">35, </v>
       </c>
@@ -3491,64 +3446,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Redusă', </v>
       </c>
-      <c r="G31" s="6" t="str">
+      <c r="G31" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Rx locală', </v>
       </c>
-      <c r="H31" s="5" t="str">
+      <c r="H31" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Radiografie (radiologie dentară)', </v>
       </c>
-      <c r="I31" s="6" t="str">
+      <c r="I31" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J31" s="6" t="str">
+      <c r="J31" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Film_radiografic_sau_digital"}', </v>
       </c>
-      <c r="K31" s="11" t="str">
+      <c r="K31" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Inhalosedare cu protoxid de azot pentru copii.jpg'),</v>
+        <v>'Radiografie locală.jpg'),</v>
       </c>
       <c r="L31" s="1"/>
-      <c r="P31" s="7" t="s">
+      <c r="P31" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="R31" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="S31" s="7" t="s">
+      <c r="R31" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="S31" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="T31" s="6" t="s">
-        <v>183</v>
+      <c r="T31" s="5" t="s">
+        <v>169</v>
       </c>
       <c r="U31" s="1" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="V31" s="1" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="W31" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="Y31" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="Y31" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="AA31" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="AB31" s="6" t="b">
+      <c r="AA31" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="AB31" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC31" s="9">
+      <c r="AC31" s="8">
         <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A32" s="7"/>
-      <c r="B32" s="8" t="str">
+      <c r="A32" s="6"/>
+      <c r="B32" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Radiografie panoramică digitală (OPG)', </v>
       </c>
@@ -3556,7 +3511,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Imagine completă a maxilarelor și dinților.', </v>
       </c>
-      <c r="D32" s="9" t="str">
+      <c r="D32" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">100, </v>
       </c>
@@ -3568,64 +3523,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G32" s="6" t="str">
+      <c r="G32" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Rx panoramică', </v>
       </c>
-      <c r="H32" s="5" t="str">
+      <c r="H32" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Radiografie (radiologie dentară)', </v>
       </c>
-      <c r="I32" s="6" t="str">
+      <c r="I32" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J32" s="6" t="str">
+      <c r="J32" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Film_panoramic_sau_digital"}', </v>
       </c>
-      <c r="K32" s="11" t="str">
+      <c r="K32" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Periaj profesional Happy Brush.jpg'),</v>
+        <v>'Radiografie panoramică digitală (OPG).jpg'),</v>
       </c>
       <c r="L32" s="1"/>
-      <c r="P32" s="7" t="s">
+      <c r="P32" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="R32" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="S32" s="7" t="s">
+      <c r="R32" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="S32" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="T32" s="6" t="s">
-        <v>184</v>
+      <c r="T32" s="5" t="s">
+        <v>170</v>
       </c>
       <c r="U32" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V32" s="1" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="W32" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="Y32" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="Y32" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="AA32" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="AB32" s="6" t="b">
+      <c r="AA32" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="AB32" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC32" s="9">
+      <c r="AC32" s="8">
         <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A33" s="7"/>
-      <c r="B33" s="8" t="str">
+      <c r="A33" s="6"/>
+      <c r="B33" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Tomografie completă maxilară/mandibulară', </v>
       </c>
@@ -3633,7 +3588,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Imagine 3D completă pentru diagnostic detaliat.', </v>
       </c>
-      <c r="D33" s="9" t="str">
+      <c r="D33" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">750, </v>
       </c>
@@ -3645,64 +3600,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G33" s="6" t="str">
+      <c r="G33" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'CT complet', </v>
       </c>
-      <c r="H33" s="5" t="str">
+      <c r="H33" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Radiografie (radiologie dentară)', </v>
       </c>
-      <c r="I33" s="6" t="str">
+      <c r="I33" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J33" s="6" t="str">
+      <c r="J33" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Tomograf", "echipamente_imagistică_3D"}', </v>
       </c>
-      <c r="K33" s="11" t="str">
+      <c r="K33" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Radiografie locală.jpg'),</v>
+        <v>'Tomografie completă maxilară/mandibulară.jpg'),</v>
       </c>
       <c r="L33" s="1"/>
-      <c r="P33" s="7" t="s">
+      <c r="P33" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R33" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="S33" s="7" t="s">
+      <c r="R33" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="S33" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="T33" s="6" t="s">
-        <v>185</v>
+      <c r="T33" s="5" t="s">
+        <v>171</v>
       </c>
       <c r="U33" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V33" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="W33" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="Y33" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="Y33" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="AA33" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="AB33" s="6" t="b">
+      <c r="AA33" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="AB33" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC33" s="9">
+      <c r="AC33" s="8">
         <v>750</v>
       </c>
     </row>
     <row r="34" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A34" s="7"/>
-      <c r="B34" s="8" t="str">
+      <c r="A34" s="6"/>
+      <c r="B34" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Tomografie parțială maxilară/mandibulară ', </v>
       </c>
@@ -3710,7 +3665,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Scanare 3D a unei zone limitate.', </v>
       </c>
-      <c r="D34" s="9" t="str">
+      <c r="D34" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">450, </v>
       </c>
@@ -3722,64 +3677,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G34" s="6" t="str">
+      <c r="G34" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'CT parțial', </v>
       </c>
-      <c r="H34" s="5" t="str">
+      <c r="H34" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Radiografie (radiologie dentară)', </v>
       </c>
-      <c r="I34" s="6" t="str">
+      <c r="I34" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J34" s="6" t="str">
+      <c r="J34" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Tomograf", "echipamente_imagistică_3D"}', </v>
       </c>
-      <c r="K34" s="11" t="str">
+      <c r="K34" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Radiografie panoramică digitală (OPG).jpg'),</v>
+        <v>'Tomografie parțială maxilară/mandibulară .jpg'),</v>
       </c>
       <c r="L34" s="1"/>
-      <c r="P34" s="7" t="s">
+      <c r="P34" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="R34" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="S34" s="7" t="s">
+      <c r="R34" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="S34" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="T34" s="6" t="s">
-        <v>186</v>
+      <c r="T34" s="5" t="s">
+        <v>172</v>
       </c>
       <c r="U34" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V34" s="1" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="W34" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="Y34" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="AA34" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="AB34" s="6" t="b">
+        <v>118</v>
+      </c>
+      <c r="Y34" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="AA34" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="AB34" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC34" s="9">
+      <c r="AC34" s="8">
         <v>450</v>
       </c>
     </row>
     <row r="35" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A35" s="7"/>
-      <c r="B35" s="8" t="str">
+      <c r="A35" s="6"/>
+      <c r="B35" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Extracție dinte monoradicular', </v>
       </c>
@@ -3787,7 +3742,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Îndepărtare dinte cu o rădăcină.', </v>
       </c>
-      <c r="D35" s="9" t="str">
+      <c r="D35" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">250, </v>
       </c>
@@ -3799,64 +3754,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G35" s="6" t="str">
+      <c r="G35" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Extracție simplă', </v>
       </c>
-      <c r="H35" s="5" t="str">
+      <c r="H35" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Chirurgie dento-alveolară', </v>
       </c>
-      <c r="I35" s="6" t="str">
+      <c r="I35" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J35" s="6" t="str">
+      <c r="J35" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Anestezic_local", "instrumente_extracție"}', </v>
       </c>
-      <c r="K35" s="11" t="str">
+      <c r="K35" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Retratament endodontic.jpg'),</v>
+        <v>'Extracție dinte monoradicular.jpg'),</v>
       </c>
       <c r="L35" s="1"/>
-      <c r="P35" s="7" t="s">
+      <c r="P35" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="R35" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="S35" s="7" t="s">
+      <c r="R35" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="S35" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="T35" s="6" t="s">
-        <v>187</v>
+      <c r="T35" s="5" t="s">
+        <v>173</v>
       </c>
       <c r="U35" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V35" s="1" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="W35" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="Y35" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y35" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="AA35" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="AB35" s="6" t="b">
+      <c r="AA35" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="AB35" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC35" s="9">
+      <c r="AC35" s="8">
         <v>250</v>
       </c>
     </row>
     <row r="36" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A36" s="7"/>
-      <c r="B36" s="8" t="str">
+      <c r="A36" s="6"/>
+      <c r="B36" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Extracție dinte pluriradicular', </v>
       </c>
@@ -3864,7 +3819,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Îndepărtare molar cu mai multe rădăcini.', </v>
       </c>
-      <c r="D36" s="9" t="str">
+      <c r="D36" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">300, </v>
       </c>
@@ -3876,64 +3831,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G36" s="6" t="str">
+      <c r="G36" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Extracție molar', </v>
       </c>
-      <c r="H36" s="5" t="str">
+      <c r="H36" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Chirurgie dento-alveolară', </v>
       </c>
-      <c r="I36" s="6" t="str">
+      <c r="I36" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J36" s="6" t="str">
+      <c r="J36" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Anestezic_local", "instrumente_extracție"}', </v>
       </c>
-      <c r="K36" s="11" t="str">
+      <c r="K36" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Rezecție apicală.jpg'),</v>
+        <v>'Extracție dinte pluriradicular.jpg'),</v>
       </c>
       <c r="L36" s="1"/>
-      <c r="P36" s="7" t="s">
+      <c r="P36" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="R36" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="S36" s="7" t="s">
+      <c r="R36" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="S36" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="T36" s="6" t="s">
-        <v>188</v>
+      <c r="T36" s="5" t="s">
+        <v>174</v>
       </c>
       <c r="U36" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V36" s="1" t="s">
-        <v>160</v>
+        <v>146</v>
       </c>
       <c r="W36" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="Y36" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="Y36" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="AA36" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="AB36" s="6" t="b">
+      <c r="AA36" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="AB36" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC36" s="9">
+      <c r="AC36" s="8">
         <v>300</v>
       </c>
     </row>
     <row r="37" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A37" s="7"/>
-      <c r="B37" s="8" t="str">
+      <c r="A37" s="6"/>
+      <c r="B37" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Extracție molar de minte', </v>
       </c>
@@ -3941,7 +3896,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Îndepărtare măsea de minte.', </v>
       </c>
-      <c r="D37" s="9" t="str">
+      <c r="D37" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">500, </v>
       </c>
@@ -3953,64 +3908,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G37" s="6" t="str">
+      <c r="G37" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Extracție minte', </v>
       </c>
-      <c r="H37" s="5" t="str">
+      <c r="H37" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Chirurgie dento-alveolară', </v>
       </c>
-      <c r="I37" s="6" t="str">
+      <c r="I37" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J37" s="6" t="str">
+      <c r="J37" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Anestezic_local", "instrumente_extracție"}', </v>
       </c>
-      <c r="K37" s="11" t="str">
+      <c r="K37" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Sigilare dentară (dinte sănătos, prevenție carii).jpg'),</v>
+        <v>'Extracție molar de minte.jpg'),</v>
       </c>
       <c r="L37" s="1"/>
-      <c r="P37" s="7" t="s">
+      <c r="P37" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="R37" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="S37" s="7" t="s">
+      <c r="R37" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="S37" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="T37" s="6" t="s">
-        <v>189</v>
+      <c r="T37" s="5" t="s">
+        <v>175</v>
       </c>
       <c r="U37" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V37" s="1" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="W37" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="Y37" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="Y37" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="AA37" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="AB37" s="6" t="b">
+      <c r="AA37" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="AB37" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC37" s="9">
+      <c r="AC37" s="8">
         <v>500</v>
       </c>
     </row>
     <row r="38" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A38" s="7"/>
-      <c r="B38" s="8" t="str">
+      <c r="A38" s="6"/>
+      <c r="B38" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Extracție dinte temporar', </v>
       </c>
@@ -4018,7 +3973,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Scoaterea unui dinte de lapte.', </v>
       </c>
-      <c r="D38" s="9" t="str">
+      <c r="D38" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">120, </v>
       </c>
@@ -4030,64 +3985,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Redusă', </v>
       </c>
-      <c r="G38" s="6" t="str">
+      <c r="G38" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Extracție temporar', </v>
       </c>
-      <c r="H38" s="5" t="str">
+      <c r="H38" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Chirurgie dento-alveolară', </v>
       </c>
-      <c r="I38" s="6" t="str">
+      <c r="I38" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J38" s="6" t="str">
+      <c r="J38" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Anestezic_local", "instrumente_extracție"}', </v>
       </c>
-      <c r="K38" s="11" t="str">
+      <c r="K38" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Tomografie completă .jpg'),</v>
+        <v>'Extracție dinte temporar.jpg'),</v>
       </c>
       <c r="L38" s="1"/>
-      <c r="P38" s="7" t="s">
+      <c r="P38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="R38" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="S38" s="7" t="s">
+      <c r="R38" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="S38" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="T38" s="6" t="s">
-        <v>190</v>
+      <c r="T38" s="5" t="s">
+        <v>176</v>
       </c>
       <c r="U38" s="1" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="V38" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="W38" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="Y38" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="Y38" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="AA38" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="AB38" s="6" t="b">
+      <c r="AA38" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="AB38" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC38" s="9">
+      <c r="AC38" s="8">
         <v>120</v>
       </c>
     </row>
     <row r="39" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A39" s="7"/>
-      <c r="B39" s="8" t="str">
+      <c r="A39" s="6"/>
+      <c r="B39" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Rezecție apicală', </v>
       </c>
@@ -4095,7 +4050,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Îndepărtarea vârfului unei rădăcini infectate.', </v>
       </c>
-      <c r="D39" s="9" t="str">
+      <c r="D39" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">400, </v>
       </c>
@@ -4107,64 +4062,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Ridicată', </v>
       </c>
-      <c r="G39" s="6" t="str">
+      <c r="G39" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Rezecție apicală', </v>
       </c>
-      <c r="H39" s="5" t="str">
+      <c r="H39" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Chirurgie dento-alveolară', </v>
       </c>
-      <c r="I39" s="6" t="str">
+      <c r="I39" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J39" s="6" t="str">
+      <c r="J39" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Instrumente_chirurgicale", "anestezic", "material_sutură"}', </v>
       </c>
-      <c r="K39" s="11" t="str">
+      <c r="K39" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Tomografie parțială  .jpg'),</v>
+        <v>'Rezecție apicală.jpg'),</v>
       </c>
       <c r="L39" s="1"/>
-      <c r="P39" s="7" t="s">
+      <c r="P39" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="R39" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="S39" s="7" t="s">
+      <c r="R39" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="S39" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="T39" s="6" t="s">
+      <c r="T39" s="5" t="s">
         <v>67</v>
       </c>
       <c r="U39" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="V39" s="1" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="W39" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="Y39" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="Y39" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="AA39" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="AB39" s="6" t="b">
+      <c r="AA39" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="AB39" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC39" s="9">
+      <c r="AC39" s="8">
         <v>400</v>
       </c>
     </row>
     <row r="40" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A40" s="7"/>
-      <c r="B40" s="8" t="str">
+      <c r="A40" s="6"/>
+      <c r="B40" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Drenaj abces', </v>
       </c>
@@ -4172,7 +4127,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Eliminarea puroiului dintr-o infecție.', </v>
       </c>
-      <c r="D40" s="9" t="str">
+      <c r="D40" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">100, </v>
       </c>
@@ -4184,64 +4139,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G40" s="6" t="str">
+      <c r="G40" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Drenaj abces', </v>
       </c>
-      <c r="H40" s="5" t="str">
+      <c r="H40" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Chirurgie dento-alveolară', </v>
       </c>
-      <c r="I40" s="6" t="str">
+      <c r="I40" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J40" s="6" t="str">
+      <c r="J40" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Instrumente_chirurgicale", "drenuri", "anestezic"}', </v>
       </c>
-      <c r="K40" s="11" t="str">
+      <c r="K40" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Tratament carie dentară (obturatie).jpg'),</v>
+        <v>'Drenaj abces.jpg'),</v>
       </c>
       <c r="L40" s="1"/>
-      <c r="P40" s="7" t="s">
+      <c r="P40" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="R40" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="S40" s="7" t="s">
+      <c r="R40" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="S40" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="T40" s="6" t="s">
+      <c r="T40" s="5" t="s">
         <v>69</v>
       </c>
       <c r="U40" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V40" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="W40" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="Y40" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="Y40" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="AA40" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="AB40" s="6" t="b">
+      <c r="AA40" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="AB40" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC40" s="9">
+      <c r="AC40" s="8">
         <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A41" s="7"/>
-      <c r="B41" s="8" t="str">
+      <c r="A41" s="6"/>
+      <c r="B41" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Consultație stomatologie pediatrică', </v>
       </c>
@@ -4249,7 +4204,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Verificare orală pentru copii.', </v>
       </c>
-      <c r="D41" s="9" t="str">
+      <c r="D41" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">200, </v>
       </c>
@@ -4261,64 +4216,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Redusă', </v>
       </c>
-      <c r="G41" s="6" t="str">
+      <c r="G41" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Consult copil', </v>
       </c>
-      <c r="H41" s="5" t="str">
+      <c r="H41" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Stomatologie pediatrică', </v>
       </c>
-      <c r="I41" s="6" t="str">
+      <c r="I41" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J41" s="6" t="str">
+      <c r="J41" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Echipamente_evaluare"}', </v>
       </c>
-      <c r="K41" s="11" t="str">
+      <c r="K41" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Tratament cu alignere aparat dentar invizibil INVISALIGN Teen.jpg'),</v>
+        <v>'Consultație stomatologie pediatrică.jpg'),</v>
       </c>
       <c r="L41" s="1"/>
-      <c r="P41" s="7" t="s">
+      <c r="P41" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="R41" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="S41" s="7" t="s">
+      <c r="R41" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="S41" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="T41" s="6" t="s">
-        <v>191</v>
+      <c r="T41" s="5" t="s">
+        <v>177</v>
       </c>
       <c r="U41" s="1" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="V41" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="W41" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Y41" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="Y41" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="AA41" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="AB41" s="6" t="b">
+      <c r="AA41" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="AB41" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC41" s="9">
+      <c r="AC41" s="8">
         <v>200</v>
       </c>
     </row>
     <row r="42" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A42" s="7"/>
-      <c r="B42" s="8" t="str">
+      <c r="A42" s="6"/>
+      <c r="B42" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Consultație pedodontică de specialitate', </v>
       </c>
@@ -4326,7 +4281,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Evaluare detaliată la specialist pentru copii.', </v>
       </c>
-      <c r="D42" s="9" t="str">
+      <c r="D42" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">250, </v>
       </c>
@@ -4338,64 +4293,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G42" s="6" t="str">
+      <c r="G42" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Pedodont special', </v>
       </c>
-      <c r="H42" s="5" t="str">
+      <c r="H42" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Stomatologie pediatrică', </v>
       </c>
-      <c r="I42" s="6" t="str">
+      <c r="I42" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J42" s="6" t="str">
+      <c r="J42" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Echipamente_evaluare"}', </v>
       </c>
-      <c r="K42" s="11" t="str">
+      <c r="K42" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Tratament cu alignere aparat INVISALIGN LITE.jpg'),</v>
+        <v>'Consultație pedodontică de specialitate.jpg'),</v>
       </c>
       <c r="L42" s="1"/>
-      <c r="P42" s="7" t="s">
+      <c r="P42" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="R42" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="S42" s="7" t="s">
+      <c r="R42" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="S42" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="T42" s="6" t="s">
-        <v>192</v>
+      <c r="T42" s="5" t="s">
+        <v>178</v>
       </c>
       <c r="U42" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="V42" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="W42" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="Y42" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="AA42" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="V42" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="W42" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Y42" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="AA42" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="AB42" s="6" t="b">
+      <c r="AB42" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC42" s="9">
+      <c r="AC42" s="8">
         <v>250</v>
       </c>
     </row>
     <row r="43" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A43" s="7"/>
-      <c r="B43" s="8" t="str">
+      <c r="A43" s="6"/>
+      <c r="B43" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Anestezie locală computerizată DentaPen / sedinta ', </v>
       </c>
@@ -4403,7 +4358,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Anestezie precisă și confortabilă.', </v>
       </c>
-      <c r="D43" s="9" t="str">
+      <c r="D43" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">90, </v>
       </c>
@@ -4415,64 +4370,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Redusă', </v>
       </c>
-      <c r="G43" s="6" t="str">
+      <c r="G43" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Anestezie digitală', </v>
       </c>
-      <c r="H43" s="5" t="str">
+      <c r="H43" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Stomatologie pediatrică', </v>
       </c>
-      <c r="I43" s="6" t="str">
+      <c r="I43" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J43" s="6" t="str">
+      <c r="J43" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Dispozitiv_DentaPen", "anestezic"}', </v>
       </c>
-      <c r="K43" s="11" t="str">
+      <c r="K43" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Tratament endodontic dinte monoradicular​.jpg'),</v>
+        <v>'Anestezie locală computerizată DentaPen / sedinta .jpg'),</v>
       </c>
       <c r="L43" s="1"/>
-      <c r="P43" s="7" t="s">
+      <c r="P43" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="R43" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="R43" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="S43" s="7" t="s">
+      <c r="S43" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="T43" s="6" t="s">
-        <v>193</v>
+      <c r="T43" s="5" t="s">
+        <v>179</v>
       </c>
       <c r="U43" s="1" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="V43" s="1" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="W43" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y43" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="AA43" s="6" t="s">
-        <v>235</v>
-      </c>
-      <c r="AB43" s="6" t="b">
+        <v>127</v>
+      </c>
+      <c r="Y43" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="AA43" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="AB43" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC43" s="9">
+      <c r="AC43" s="8">
         <v>90</v>
       </c>
     </row>
     <row r="44" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A44" s="7"/>
-      <c r="B44" s="8" t="str">
+      <c r="A44" s="6"/>
+      <c r="B44" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Inhalosedare cu protoxid de azot pentru copii / ședință', </v>
       </c>
@@ -4480,7 +4435,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Relaxare ușoară pentru copii anxioși.', </v>
       </c>
-      <c r="D44" s="9" t="str">
+      <c r="D44" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">450, </v>
       </c>
@@ -4492,64 +4447,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G44" s="6" t="str">
+      <c r="G44" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Inhalosedare copil', </v>
       </c>
-      <c r="H44" s="5" t="str">
+      <c r="H44" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Stomatologie pediatrică', </v>
       </c>
-      <c r="I44" s="6" t="str">
+      <c r="I44" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J44" s="6" t="str">
+      <c r="J44" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Echipamente_inhalosedare", "protoxid_de_azot"}', </v>
       </c>
-      <c r="K44" s="11" t="str">
+      <c r="K44" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Tratament endodontic dinte pluriradicular.jpg'),</v>
+        <v>'Inhalosedare cu protoxid de azot pentru copii / ședință.jpg'),</v>
       </c>
       <c r="L44" s="1"/>
-      <c r="P44" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="R44" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="S44" s="7" t="s">
+      <c r="P44" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="R44" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="S44" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="T44" s="6" t="s">
-        <v>194</v>
+      <c r="T44" s="5" t="s">
+        <v>180</v>
       </c>
       <c r="U44" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V44" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="W44" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="Y44" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="AA44" s="6" t="s">
-        <v>236</v>
-      </c>
-      <c r="AB44" s="6" t="b">
+        <v>128</v>
+      </c>
+      <c r="Y44" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="AA44" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="AB44" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC44" s="9">
+      <c r="AC44" s="8">
         <v>450</v>
       </c>
     </row>
     <row r="45" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A45" s="7"/>
-      <c r="B45" s="8" t="str">
+      <c r="A45" s="6"/>
+      <c r="B45" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Sigilare dentară (dinte sănătos, prevenție carii)/dinte ', </v>
       </c>
@@ -4557,7 +4512,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Protecție împotriva cariilor pentru dinți sănătoși.', </v>
       </c>
-      <c r="D45" s="9" t="str">
+      <c r="D45" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">150, </v>
       </c>
@@ -4569,64 +4524,64 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Redusă', </v>
       </c>
-      <c r="G45" s="6" t="str">
+      <c r="G45" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Sigilare carii', </v>
       </c>
-      <c r="H45" s="5" t="str">
+      <c r="H45" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Stomatologie pediatrică', </v>
       </c>
-      <c r="I45" s="6" t="str">
+      <c r="I45" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">FALSE, </v>
       </c>
-      <c r="J45" s="6" t="str">
+      <c r="J45" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"Materiale_sigilante", "aplicatoare"}', </v>
       </c>
-      <c r="K45" s="11" t="str">
+      <c r="K45" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Tratament endodontic premolar.jpg'),</v>
+        <v>'Sigilare dentară (dinte sănătos, prevenție carii)/dinte .jpg'),</v>
       </c>
       <c r="L45" s="1"/>
-      <c r="P45" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="R45" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="S45" s="7" t="s">
+      <c r="P45" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="R45" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="S45" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="T45" s="6" t="s">
-        <v>195</v>
+      <c r="T45" s="5" t="s">
+        <v>181</v>
       </c>
       <c r="U45" s="1" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="V45" s="1" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="W45" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="Y45" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="AA45" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="AB45" s="6" t="b">
+        <v>129</v>
+      </c>
+      <c r="Y45" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA45" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="AB45" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="AC45" s="9">
+      <c r="AC45" s="8">
         <v>150</v>
       </c>
     </row>
     <row r="46" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A46" s="7"/>
-      <c r="B46" s="8" t="str">
+      <c r="A46" s="6"/>
+      <c r="B46" s="7" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">('Tratament carie dentară (obturatie)/dinte ', </v>
       </c>
@@ -4634,7 +4589,7 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve">'Curățare și plombare carie dentară.', </v>
       </c>
-      <c r="D46" s="9" t="str">
+      <c r="D46" s="8" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">250, </v>
       </c>
@@ -4646,58 +4601,58 @@
         <f t="shared" si="4"/>
         <v xml:space="preserve">'Medie', </v>
       </c>
-      <c r="G46" s="6" t="str">
+      <c r="G46" s="5" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">'Plombă dentară', </v>
       </c>
-      <c r="H46" s="5" t="str">
+      <c r="H46" s="4" t="str">
         <f t="shared" si="6"/>
         <v xml:space="preserve">'Stomatologie pediatrică', </v>
       </c>
-      <c r="I46" s="6" t="str">
+      <c r="I46" s="5" t="str">
         <f t="shared" si="7"/>
         <v xml:space="preserve">TRUE, </v>
       </c>
-      <c r="J46" s="6" t="str">
+      <c r="J46" s="5" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">'{"compozit", "amalgam", "fotopolimerizabil"}', </v>
       </c>
-      <c r="K46" s="11" t="str">
+      <c r="K46" s="10" t="str">
         <f t="shared" si="9"/>
-        <v>'Utilizarea microscopului ​.jpg'),</v>
+        <v>'Tratament carie dentară (obturatie)/dinte .jpg'),</v>
       </c>
       <c r="L46" s="1"/>
-      <c r="P46" s="7" t="s">
+      <c r="P46" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="R46" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="S46" s="7" t="s">
+      <c r="R46" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="S46" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="T46" s="6" t="s">
-        <v>196</v>
+      <c r="T46" s="5" t="s">
+        <v>182</v>
       </c>
       <c r="U46" s="1" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V46" s="1" t="s">
-        <v>160</v>
+        <v>146</v>
       </c>
       <c r="W46" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="Y46" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="AA46" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="AB46" s="6" t="b">
+        <v>130</v>
+      </c>
+      <c r="Y46" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="AA46" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="AB46" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="AC46" s="9">
+      <c r="AC46" s="8">
         <v>250</v>
       </c>
     </row>
@@ -4712,5 +4667,6 @@
     <sortCondition ref="R1:R55"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>